<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:34:04)
</commit_message>
<xml_diff>
--- a/qayta_tekshiruv/Talabalar_Yangilangan_Royxat.xlsx
+++ b/qayta_tekshiruv/Talabalar_Yangilangan_Royxat.xlsx
@@ -17317,7 +17317,11 @@
           <t>AD1671106</t>
         </is>
       </c>
-      <c r="K150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>60906055720101</t>
+        </is>
+      </c>
       <c r="L150" s="5" t="inlineStr">
         <is>
           <t>18.08.2022</t>
@@ -17328,7 +17332,11 @@
           <t>09.06.2005</t>
         </is>
       </c>
-      <c r="N150" s="5" t="inlineStr"/>
+      <c r="N150" s="5" t="inlineStr">
+        <is>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
       <c r="O150" s="4" t="inlineStr"/>
       <c r="P150" s="2" t="inlineStr"/>
       <c r="Q150" s="4" t="inlineStr"/>
@@ -28775,7 +28783,11 @@
           <t>AD1671106</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>60906055720101</t>
+        </is>
+      </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
           <t>18.08.2022</t>
@@ -28786,7 +28798,11 @@
           <t>09.06.2005</t>
         </is>
       </c>
-      <c r="N26" s="5" t="inlineStr"/>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
       <c r="O26" s="4" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:38:35)
</commit_message>
<xml_diff>
--- a/qayta_tekshiruv/Talabalar_Yangilangan_Royxat.xlsx
+++ b/qayta_tekshiruv/Talabalar_Yangilangan_Royxat.xlsx
@@ -18245,11 +18245,23 @@
         </is>
       </c>
       <c r="O158" s="4" t="inlineStr"/>
-      <c r="P158" s="2" t="inlineStr"/>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>UM+0862565</t>
+        </is>
+      </c>
       <c r="Q158" s="4" t="inlineStr"/>
-      <c r="R158" s="4" t="inlineStr"/>
+      <c r="R158" s="4" t="inlineStr">
+        <is>
+          <t>1-sonli+ayrim+fanlar+chuqur+o'rganiladigan+ixtisoslashtirilgan+maktab</t>
+        </is>
+      </c>
       <c r="S158" s="5" t="inlineStr"/>
-      <c r="T158" s="5" t="inlineStr"/>
+      <c r="T158" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="U158" s="16" t="inlineStr">
         <is>
           <t>CHALA</t>
@@ -32584,11 +32596,23 @@
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>UM+0862565</t>
+        </is>
+      </c>
       <c r="Q26" s="4" t="inlineStr"/>
-      <c r="R26" s="4" t="inlineStr"/>
+      <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>1-sonli+ayrim+fanlar+chuqur+o'rganiladigan+ixtisoslashtirilgan+maktab</t>
+        </is>
+      </c>
       <c r="S26" s="5" t="inlineStr"/>
-      <c r="T26" s="5" t="inlineStr"/>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="U26" s="16" t="inlineStr">
         <is>
           <t>CHALA</t>

</xml_diff>

<commit_message>
Loyiha tuzilmasi: papkalarga ajratish va yangi web (web/) asosiy portal
- Ildizda faqat .bat va texnik fayllar; qolganlari vazifasiga qarab:
  data/ (baza), hujjatlar/ (shartnomalar), hisobotlar/, xizmatlar/,
  eski_portal/ (arxiv), arxiv/
- Barcha Python skriptlari, xizmatlar va web yangi yo'llarga moslandi
- Vercel api/*.js web/ ga ko'chirildi: /api/telegram_webhook, /api/view_group_pdf
- Qabul shabloni: rasmiy EN/RU tarjima (web/lib/qabul.ts), "Guruhi" ustuni,
  portal eksporti Python bilan bir xil; hujjat rasmini joyida zoom qilish
- 26-07 guruhi olib tashlandi (talaba 26-03 ga o'tkazildi)
- Shubhali ma'lumotlar tekshiruvi va docx'dan telefonlar skriptlari

Vercel: Root Directory = web

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qayta_tekshiruv/Talabalar_Yangilangan_Royxat.xlsx
+++ b/qayta_tekshiruv/Talabalar_Yangilangan_Royxat.xlsx
@@ -14,19 +14,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26-04 (Hamdamova.M)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26-05 (Rayimova.X)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26-06 (Yuldashev.O)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26-07 (Asraliyev.A)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safdan chiqarilganlar" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safdan chiqarilganlar" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jami'!$A$1:$X$179</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'26-01 (Mirzayeva.D)'!$A$1:$X$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'26-02 (Ochilov.D)'!$A$1:$X$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'26-03 (To''rayeva.S)'!$A$1:$X$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'26-03 (To''rayeva.S)'!$A$1:$X$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'26-04 (Hamdamova.M)'!$A$1:$X$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'26-05 (Rayimova.X)'!$A$1:$X$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'26-06 (Yuldashev.O)'!$A$1:$X$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'26-07 (Asraliyev.A)'!$A$1:$X$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Safdan chiqarilganlar'!$A$1:$X$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Safdan chiqarilganlar'!$A$1:$X$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9626,7 +9624,7 @@
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-03</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -26019,7 +26017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X33"/>
+  <dimension ref="A1:X34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -27041,74 +27039,78 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Mustafayeva Madina</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
+          <t>Murtazayeva Kamola</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07 00:00:00</t>
+          <t>2026-06-29 00:00:00</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Ortiq qizi</t>
+          <t>Jamoliddin qizi</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Mustafayeva Madina Ortiq qizi</t>
+          <t>Murtazayeva Kamola Jamoliddin qizi</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Mustafayeva Madina Ortiq qizi</t>
+          <t>Murtazayeva Kamola Jamoliddin qizi</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>AE4846447</t>
+          <t>AC1458884</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>63110085680103</t>
+          <t>42708915590028</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>04.11.2018</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>31.10.2008</t>
+          <t>27.08.1991</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>Kitob tumani</t>
+          <t>Shahrisabz tumani</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>Mustafayeva Madina Ortiq qizi</t>
+          <t>Murtazayeva Kamola Jamoliddin qizi</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>UM 03729407</t>
+          <t>O'r-Sh 0987579</t>
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr"/>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t>49-maktab</t>
+          <t>Ixtisoslashgan maktab</t>
         </is>
       </c>
       <c r="S10" s="5" t="inlineStr">
@@ -27116,10 +27118,8 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
+      <c r="T10" s="5" t="n">
+        <v>2009</v>
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
@@ -27128,7 +27128,7 @@
       </c>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>Mustafayeva Madina Ortiq qizi (#282) ma'lumotlari tasdiqlandi</t>
+          <t>Otasining ismi 'Jamoliddin qizi' deb to'g'rilandi (#25)</t>
         </is>
       </c>
       <c r="W10" s="8" t="inlineStr">
@@ -27153,66 +27153,74 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Niyozova Komila</t>
+          <t>Mustafayeva Madina</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr"/>
-      <c r="E11" s="12" t="inlineStr"/>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>282</t>
+        </is>
+      </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>2026-09-17 00:00:00</t>
+          <t>2026-09-07 00:00:00</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Toshpulatovna</t>
+          <t>Ortiq qizi</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Niyozova Komila Toshpulatovna</t>
+          <t>Mustafayeva Madina Ortiq qizi</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>Niyozova Komila Toshpulatovna</t>
+          <t>Mustafayeva Madina Ortiq qizi</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>AB9205278</t>
+          <t>AE4846447</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>42405832640057</t>
+          <t>63110085680103</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>07.04.2018</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>24.05.1983</t>
-        </is>
-      </c>
-      <c r="N11" s="12" t="inlineStr"/>
+          <t>31.10.2008</t>
+        </is>
+      </c>
+      <c r="N11" s="12" t="inlineStr">
+        <is>
+          <t>Kitob tumani</t>
+        </is>
+      </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>Niyozova Komila Toshpulatovna</t>
+          <t>Mustafayeva Madina Ortiq qizi</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>DB 00222382</t>
+          <t>UM 03729407</t>
         </is>
       </c>
       <c r="Q11" s="11" t="inlineStr"/>
       <c r="R11" s="11" t="inlineStr">
         <is>
-          <t>Qashqadaryo viloyati Kitob tumani 21-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>49-maktab</t>
         </is>
       </c>
       <c r="S11" s="12" t="inlineStr">
@@ -27222,7 +27230,7 @@
       </c>
       <c r="T11" s="12" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -27232,7 +27240,7 @@
       </c>
       <c r="V11" s="11" t="inlineStr">
         <is>
-          <t>Telegram (tg) orqali yuborilgan pasport va shahodatnoma dublikatidan to'liq kiritildi</t>
+          <t>Mustafayeva Madina Ortiq qizi (#282) ma'lumotlari tasdiqlandi</t>
         </is>
       </c>
       <c r="W11" s="8" t="inlineStr">
@@ -27240,9 +27248,9 @@
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X11" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X11" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27257,82 +27265,66 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Norboboyeva Farangiz</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
-      </c>
+          <t>Niyozova Komila</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-02 00:00:00</t>
+          <t>2026-09-17 00:00:00</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Nuriddin qizi</t>
+          <t>Toshpulatovna</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Norboboyeva Farangiz Nuriddin qizi</t>
+          <t>Niyozova Komila Toshpulatovna</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Norboboyeva Farangiz Nuriddin qizi</t>
+          <t>Niyozova Komila Toshpulatovna</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>AE5898909</t>
+          <t>AB9205278</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>62808085590100</t>
+          <t>42405832640057</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>16.01.2026</t>
+          <t>07.04.2018</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>28.08.2008</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>Shahrisabz tumani</t>
-        </is>
-      </c>
+          <t>24.05.1983</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>Norboboyeva Farangiz Nuriddin qizi</t>
+          <t>Niyozova Komila Toshpulatovna</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>UM 03753862</t>
-        </is>
-      </c>
-      <c r="Q12" s="4" t="inlineStr">
-        <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3372975/3160794/4c79322b-c376-4475-b3c0-ade80431cd1f?preview=true</t>
-        </is>
-      </c>
+          <t>DB 00222382</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>19-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Qashqadaryo viloyati Kitob tumani 21-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S12" s="5" t="inlineStr">
@@ -27342,7 +27334,7 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="U12" s="7" t="inlineStr">
@@ -27350,15 +27342,19 @@
           <t>TOPILDI</t>
         </is>
       </c>
-      <c r="V12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>Telegram (tg) orqali yuborilgan pasport va shahodatnoma dublikatidan to'liq kiritildi</t>
+        </is>
+      </c>
       <c r="W12" s="8" t="inlineStr">
         <is>
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
-      <c r="X12" s="7" t="inlineStr">
-        <is>
-          <t>TASDIQLANDI</t>
+      <c r="X12" s="16" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>
@@ -27373,7 +27369,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Pardaqulova Farzona</t>
+          <t>Norboboyeva Farangiz</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -27383,7 +27379,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>231</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
@@ -27393,37 +27389,37 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Shovkatovna</t>
+          <t>Nuriddin qizi</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Pardaqulova Farzona Shovkatovna</t>
+          <t>Norboboyeva Farangiz Nuriddin qizi</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>Pardaqulova Farzona Shovkatovna</t>
+          <t>Norboboyeva Farangiz Nuriddin qizi</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>AE1336538</t>
+          <t>AE5898909</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>60312085590052</t>
+          <t>62808085590100</t>
         </is>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>23.01.2025</t>
+          <t>16.01.2026</t>
         </is>
       </c>
       <c r="M13" s="12" t="inlineStr">
         <is>
-          <t>03.12.2008</t>
+          <t>28.08.2008</t>
         </is>
       </c>
       <c r="N13" s="12" t="inlineStr">
@@ -27433,22 +27429,22 @@
       </c>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>Pardaqulova Farzona Shovkatovna</t>
+          <t>Norboboyeva Farangiz Nuriddin qizi</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>UM 03755343</t>
+          <t>UM 03753862</t>
         </is>
       </c>
       <c r="Q13" s="11" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4019179/3526276/61dfdf8f-87f2-4595-8ec2-b9d8efc6be60?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3372975/3160794/4c79322b-c376-4475-b3c0-ade80431cd1f?preview=true</t>
         </is>
       </c>
       <c r="R13" s="11" t="inlineStr">
         <is>
-          <t>61-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>19-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S13" s="12" t="inlineStr">
@@ -27469,7 +27465,7 @@
       <c r="V13" s="11" t="inlineStr"/>
       <c r="W13" s="8" t="inlineStr">
         <is>
-          <t>Pasport: MOS</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="X13" s="7" t="inlineStr">
@@ -27489,7 +27485,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Pardayeva Farangiz</t>
+          <t>Pardaqulova Farzona</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -27499,7 +27495,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>90</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -27509,37 +27505,37 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Norali qizi</t>
+          <t>Shovkatovna</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Pardayeva Farangiz Norali qizi</t>
+          <t>Pardaqulova Farzona Shovkatovna</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Pardayeva Farangiz Norali qizi</t>
+          <t>Pardaqulova Farzona Shovkatovna</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>AE5643897</t>
+          <t>AE1336538</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>60102085590053</t>
+          <t>60312085590052</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>29.12.2025</t>
+          <t>23.01.2025</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>01.02.2008</t>
+          <t>03.12.2008</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -27549,22 +27545,22 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>Pardayeva Farangiz Norali qizi</t>
+          <t>Pardaqulova Farzona Shovkatovna</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>UM 03755453</t>
+          <t>UM 03755343</t>
         </is>
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4199408/3752037/081f6da6-bd38-4be6-8cb8-5e771f5a7a10?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4019179/3526276/61dfdf8f-87f2-4595-8ec2-b9d8efc6be60?preview=true</t>
         </is>
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
-          <t>68-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>61-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S14" s="5" t="inlineStr">
@@ -27585,7 +27581,7 @@
       <c r="V14" s="4" t="inlineStr"/>
       <c r="W14" s="8" t="inlineStr">
         <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+          <t>Pasport: MOS</t>
         </is>
       </c>
       <c r="X14" s="7" t="inlineStr">
@@ -27605,7 +27601,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Primova Husnora</t>
+          <t>Pardayeva Farangiz</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -27615,7 +27611,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>105</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -27625,37 +27621,37 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Shovkat qizi</t>
+          <t>Norali qizi</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Primova Husnora Shovkat qizi</t>
+          <t>Pardayeva Farangiz Norali qizi</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>Primova Husnora Shovkat qizi</t>
+          <t>Pardayeva Farangiz Norali qizi</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>AC 0443770</t>
+          <t>AE5643897</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>61310015590029</t>
+          <t>60102085590053</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>10.12.2018</t>
+          <t>29.12.2025</t>
         </is>
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>13.10.2001</t>
+          <t>01.02.2008</t>
         </is>
       </c>
       <c r="N15" s="12" t="inlineStr">
@@ -27663,37 +27659,45 @@
           <t>Shahrisabz tumani</t>
         </is>
       </c>
-      <c r="O15" s="11" t="inlineStr"/>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>Pardayeva Farangiz Norali qizi</t>
+        </is>
+      </c>
       <c r="P15" s="9" t="inlineStr">
         <is>
-          <t>D 0095067</t>
-        </is>
-      </c>
-      <c r="Q15" s="11" t="inlineStr"/>
+          <t>UM 03755453</t>
+        </is>
+      </c>
+      <c r="Q15" s="11" t="inlineStr">
+        <is>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4199408/3752037/081f6da6-bd38-4be6-8cb8-5e771f5a7a10?preview=true</t>
+        </is>
+      </c>
       <c r="R15" s="11" t="inlineStr">
         <is>
-          <t>Shahrisabz texnalogiya kasb-hunar kolleji</t>
+          <t>68-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S15" s="12" t="inlineStr">
         <is>
-          <t>Diplom</t>
+          <t>Shahodatnoma</t>
         </is>
       </c>
       <c r="T15" s="12" t="inlineStr">
         <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="U15" s="17" t="inlineStr">
-        <is>
-          <t>FAYL_YOQ</t>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U15" s="7" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
         </is>
       </c>
       <c r="V15" s="11" t="inlineStr"/>
-      <c r="W15" s="15" t="inlineStr">
-        <is>
-          <t>TEKSHIRILMAGAN</t>
+      <c r="W15" s="8" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="X15" s="7" t="inlineStr">
@@ -27713,7 +27717,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Rasulova Husnobod</t>
+          <t>Primova Husnora</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -27723,7 +27727,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>392</t>
+          <t>251</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -27733,83 +27737,75 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Bekmurod qizi</t>
+          <t>Shovkat qizi</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Rasulova Husnobod Bekmurod qizi</t>
+          <t>Primova Husnora Shovkat qizi</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Rasulova Husnobod Bekmurod qizi</t>
+          <t>Primova Husnora Shovkat qizi</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>AD1615363</t>
+          <t>AC 0443770</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>62705055720049</t>
+          <t>61310015590029</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>03.08.2022</t>
+          <t>10.12.2018</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>27.05.2005</t>
+          <t>13.10.2001</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Chiroqchi tumani</t>
-        </is>
-      </c>
-      <c r="O16" s="4" t="inlineStr">
-        <is>
-          <t>Rasulova Husnobod Bekmurod qizi</t>
-        </is>
-      </c>
+          <t>Shahrisabz tumani</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>UM 01891815</t>
+          <t>D 0095067</t>
         </is>
       </c>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>49-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Shahrisabz texnalogiya kasb-hunar kolleji</t>
         </is>
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="U16" s="7" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
-        </is>
-      </c>
-      <c r="V16" s="4" t="inlineStr">
-        <is>
-          <t>KARANTIN: ❌ Bir xil Shahodatnoma (UM 01891815) 2 ta talabada: Suyunova Maftuna [26-02], Rasulova Husnobod [26-03]; ❌ Bir xil QR havola (https://e-shahodatnoma.uz/api/public/getcertpdf/921114/889651/0cca6b2c-74dd-4711-d168-08db6f99367e?preview=true) 2 ta talaba</t>
-        </is>
-      </c>
-      <c r="W16" s="8" t="inlineStr">
-        <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="U16" s="17" t="inlineStr">
+        <is>
+          <t>FAYL_YOQ</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="15" t="inlineStr">
+        <is>
+          <t>TEKSHIRILMAGAN</t>
         </is>
       </c>
       <c r="X16" s="7" t="inlineStr">
@@ -27829,7 +27825,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Rayimova Nozliya</t>
+          <t>Rasulova Husnobod</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -27839,60 +27835,68 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>392</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>2026-09-08 00:00:00</t>
+          <t>2026-09-02 00:00:00</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>Laziz qizi</t>
+          <t>Bekmurod qizi</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>Rayimova Nozliya Laziz qizi</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="inlineStr"/>
+          <t>Rasulova Husnobod Bekmurod qizi</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>Rasulova Husnobod Bekmurod qizi</t>
+        </is>
+      </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>AE4759683</t>
+          <t>AD1615363</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>62606085590056</t>
+          <t>62705055720049</t>
         </is>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>03.08.2022</t>
         </is>
       </c>
       <c r="M17" s="12" t="inlineStr">
         <is>
-          <t>26.06.2008</t>
+          <t>27.05.2005</t>
         </is>
       </c>
       <c r="N17" s="12" t="inlineStr">
         <is>
-          <t>Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="O17" s="11" t="inlineStr"/>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>Rasulova Husnobod Bekmurod qizi</t>
+        </is>
+      </c>
       <c r="P17" s="9" t="inlineStr">
         <is>
-          <t>UM 03755475</t>
+          <t>UM 01891815</t>
         </is>
       </c>
       <c r="Q17" s="11" t="inlineStr"/>
       <c r="R17" s="11" t="inlineStr">
         <is>
-          <t>68-maktab</t>
+          <t>49-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S17" s="12" t="inlineStr">
@@ -27902,18 +27906,22 @@
       </c>
       <c r="T17" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="U17" s="17" t="inlineStr">
-        <is>
-          <t>FAYL_YOQ</t>
-        </is>
-      </c>
-      <c r="V17" s="11" t="inlineStr"/>
-      <c r="W17" s="15" t="inlineStr">
-        <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="U17" s="7" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V17" s="11" t="inlineStr">
+        <is>
+          <t>KARANTIN: ❌ Bir xil Shahodatnoma (UM 01891815) 2 ta talabada: Suyunova Maftuna [26-02], Rasulova Husnobod [26-03]; ❌ Bir xil QR havola (https://e-shahodatnoma.uz/api/public/getcertpdf/921114/889651/0cca6b2c-74dd-4711-d168-08db6f99367e?preview=true) 2 ta talaba</t>
+        </is>
+      </c>
+      <c r="W17" s="8" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="X17" s="7" t="inlineStr">
@@ -27933,78 +27941,70 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Rustamova Charos</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
+          <t>Rayimova Nozliya</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>291</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15 00:00:00</t>
+          <t>2026-09-08 00:00:00</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>O'ktam qizi</t>
+          <t>Laziz qizi</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Rustamova Charos O'ktam qizi</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Rustamova Charos O'ktam qizi</t>
-        </is>
-      </c>
+          <t>Rayimova Nozliya Laziz qizi</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>AE4730990</t>
+          <t>AE4759683</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>60810085680017</t>
+          <t>62606085590056</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>22.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>08.10.2008</t>
+          <t>26.06.2008</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>Kitob tumani</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="inlineStr">
-        <is>
-          <t>Rustamova Charos O'ktam qizi</t>
-        </is>
-      </c>
+          <t>Shahrisabz tumani</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>UM 03728038</t>
-        </is>
-      </c>
-      <c r="Q18" s="4" t="inlineStr">
-        <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4065248/3579915/251a81e0-79f2-4882-bc82-231a0a1ab956?preview=true</t>
-        </is>
-      </c>
+          <t>UM 03755475</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>4-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>68-maktab</t>
         </is>
       </c>
       <c r="S18" s="5" t="inlineStr">
@@ -28012,22 +28012,20 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T18" s="5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="U18" s="7" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
-        </is>
-      </c>
-      <c r="V18" s="4" t="inlineStr">
-        <is>
-          <t>Telegram (tg) orqali yuborilgan haqiqiy ID-karta va Shahodatnoma rasmlari biriktirildi</t>
-        </is>
-      </c>
-      <c r="W18" s="8" t="inlineStr">
-        <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U18" s="17" t="inlineStr">
+        <is>
+          <t>FAYL_YOQ</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="15" t="inlineStr">
+        <is>
+          <t>TEKSHIRILMAGAN</t>
         </is>
       </c>
       <c r="X18" s="7" t="inlineStr">
@@ -28047,88 +28045,106 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Salayeva Dilroz</t>
+          <t>Rustamova Charos</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr"/>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>309</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>2026-09-02 00:00:00</t>
+          <t>2026-09-15 00:00:00</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>Muroulla qizi</t>
+          <t>O'ktam qizi</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>Salayeva Dilroz Muroulla qizi</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr"/>
+          <t>Rustamova Charos O'ktam qizi</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Rustamova Charos O'ktam qizi</t>
+        </is>
+      </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>AE3039330</t>
+          <t>AE4730990</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>60408085730030</t>
+          <t>60810085680017</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>16.06.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="M19" s="12" t="inlineStr">
         <is>
-          <t>04.08.2008</t>
+          <t>08.10.2008</t>
         </is>
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
-          <t>Yakkabog' tumani</t>
-        </is>
-      </c>
-      <c r="O19" s="11" t="inlineStr"/>
+          <t>Kitob tumani</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>Rustamova Charos O'ktam qizi</t>
+        </is>
+      </c>
       <c r="P19" s="9" t="inlineStr">
         <is>
-          <t>UM 03758292</t>
-        </is>
-      </c>
-      <c r="Q19" s="11" t="inlineStr"/>
+          <t>UM 03728038</t>
+        </is>
+      </c>
+      <c r="Q19" s="11" t="inlineStr">
+        <is>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4065248/3579915/251a81e0-79f2-4882-bc82-231a0a1ab956?preview=true</t>
+        </is>
+      </c>
       <c r="R19" s="11" t="inlineStr">
         <is>
-          <t>81-sonli umumiy o'rta ta'lim maktabi</t>
-        </is>
-      </c>
-      <c r="S19" s="12" t="inlineStr"/>
-      <c r="T19" s="12" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="U19" s="17" t="inlineStr">
-        <is>
-          <t>FAYL_YOQ</t>
-        </is>
-      </c>
-      <c r="V19" s="11" t="inlineStr"/>
-      <c r="W19" s="15" t="inlineStr">
-        <is>
-          <t>TEKSHIRILMAGAN</t>
-        </is>
-      </c>
-      <c r="X19" s="16" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+          <t>4-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
+      <c r="S19" s="12" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="T19" s="12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="U19" s="7" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V19" s="11" t="inlineStr">
+        <is>
+          <t>Telegram (tg) orqali yuborilgan haqiqiy ID-karta va Shahodatnoma rasmlari biriktirildi</t>
+        </is>
+      </c>
+      <c r="W19" s="8" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+        </is>
+      </c>
+      <c r="X19" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28143,13 +28159,13 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Sayfiyeva Zarina</t>
+          <t>Salayeva Dilroz</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>205</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -28159,88 +28175,72 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Axmad qizi</t>
+          <t>Muroulla qizi</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Sayfiyeva Zarina Axmad qizi</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Sayfiyeva Zarina Axmad qizi</t>
-        </is>
-      </c>
+          <t>Salayeva Dilroz Muroulla qizi</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr"/>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>AD7984192</t>
+          <t>AE3039330</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>61007085590081</t>
+          <t>60408085730030</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>23.07.2024</t>
+          <t>16.06.2025</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>10.07.2008</t>
+          <t>04.08.2008</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="O20" s="4" t="inlineStr">
-        <is>
-          <t>Sayfiyeva Zarina Axmad qizi</t>
-        </is>
-      </c>
+          <t>Yakkabog' tumani</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>UM 03751932</t>
-        </is>
-      </c>
-      <c r="Q20" s="4" t="inlineStr">
-        <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3832608/3447191/76c097af-86b5-43c8-a92d-2811565e56f3?preview=true</t>
-        </is>
-      </c>
+          <t>UM 03758292</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>7-sonli umumiy o'rta ta'lim maktabi</t>
-        </is>
-      </c>
-      <c r="S20" s="5" t="inlineStr">
-        <is>
-          <t>Shahodatnoma</t>
-        </is>
-      </c>
+          <t>81-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="U20" s="7" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
+      <c r="U20" s="17" t="inlineStr">
+        <is>
+          <t>FAYL_YOQ</t>
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr"/>
-      <c r="W20" s="8" t="inlineStr">
-        <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
-        </is>
-      </c>
-      <c r="X20" s="7" t="inlineStr">
-        <is>
-          <t>TASDIQLANDI</t>
+      <c r="W20" s="15" t="inlineStr">
+        <is>
+          <t>TEKSHIRILMAGAN</t>
+        </is>
+      </c>
+      <c r="X20" s="16" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>
@@ -28255,78 +28255,78 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Sayidova Dilafro'z</t>
+          <t>Sayfiyeva Zarina</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr"/>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 00:00:00</t>
+          <t>2026-09-02 00:00:00</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Qahramon qizi</t>
+          <t>Axmad qizi</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Sayidova Dilafro'z Qahramon qizi</t>
+          <t>Sayfiyeva Zarina Axmad qizi</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
-          <t>Sayidova Dilafro'z Qahramon qizi</t>
+          <t>Sayfiyeva Zarina Axmad qizi</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>AE6071273</t>
+          <t>AD7984192</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>62708095680047</t>
+          <t>61007085590081</t>
         </is>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>27.01.2026</t>
+          <t>23.07.2024</t>
         </is>
       </c>
       <c r="M21" s="12" t="inlineStr">
         <is>
-          <t>27.08.2009</t>
+          <t>10.07.2008</t>
         </is>
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
-          <t>Kitob tumani</t>
+          <t>Shahrisabz tumani</t>
         </is>
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>Sayidova Dilafro'z Qahramon qizi</t>
+          <t>Sayfiyeva Zarina Axmad qizi</t>
         </is>
       </c>
       <c r="P21" s="9" t="inlineStr">
         <is>
-          <t>UM 03729168</t>
+          <t>UM 03751932</t>
         </is>
       </c>
       <c r="Q21" s="11" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3743118/3827061/8d968761-cded-44aa-a481-f5732e7b775c?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3832608/3447191/76c097af-86b5-43c8-a92d-2811565e56f3?preview=true</t>
         </is>
       </c>
       <c r="R21" s="11" t="inlineStr">
         <is>
-          <t>38-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>7-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S21" s="12" t="inlineStr">
@@ -28367,82 +28367,78 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Shamsiyeva Fotima</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
+          <t>Sayidova Dilafro'z</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>263</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-02 00:00:00</t>
+          <t>2026-09-04 00:00:00</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Sharofiddin qizi</t>
+          <t>Qahramon qizi</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Shamsiyeva Fotima Sharofiddin qizi</t>
+          <t>Sayidova Dilafro'z Qahramon qizi</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Shamsiyeva Fotima Sharofiddin qizi</t>
+          <t>Sayidova Dilafro'z Qahramon qizi</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>AE2370999</t>
+          <t>AE6071273</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>60307085730074</t>
+          <t>62708095680047</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>17.04.2025</t>
+          <t>27.01.2026</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>03.07.2008</t>
+          <t>27.08.2009</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>Yakkabog' tumani</t>
+          <t>Kitob tumani</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>Shamsiyeva Fotima Sharofiddin qizi</t>
+          <t>Sayidova Dilafro'z Qahramon qizi</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>UM 03758004</t>
+          <t>UM 03729168</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3845467/3883533/77671008-6a79-4442-bbd3-dc2cfb091ca8?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3743118/3827061/8d968761-cded-44aa-a481-f5732e7b775c?preview=true</t>
         </is>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>69-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>38-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S22" s="5" t="inlineStr">
@@ -28483,7 +28479,7 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Shukurova Zilola</t>
+          <t>Shamsiyeva Fotima</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -28493,7 +28489,7 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>107</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
@@ -28503,63 +28499,67 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>Farxod qizi</t>
+          <t>Sharofiddin qizi</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Shukurova Zilola Farxod qizi</t>
+          <t>Shamsiyeva Fotima Sharofiddin qizi</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
-          <t>Shukurova Zilola Farxod qizi</t>
+          <t>Shamsiyeva Fotima Sharofiddin qizi</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>AE1059205</t>
+          <t>AE2370999</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>60610085590150</t>
+          <t>60307085730074</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>07.01.2025</t>
+          <t>17.04.2025</t>
         </is>
       </c>
       <c r="M23" s="12" t="inlineStr">
         <is>
-          <t>06.10.2008</t>
+          <t>03.07.2008</t>
         </is>
       </c>
       <c r="N23" s="12" t="inlineStr">
         <is>
-          <t>Shahrisabz tumani</t>
+          <t>Yakkabog' tumani</t>
         </is>
       </c>
       <c r="O23" s="11" t="inlineStr">
         <is>
-          <t>Shukurova Zilola Farhod qizi</t>
+          <t>Shamsiyeva Fotima Sharofiddin qizi</t>
         </is>
       </c>
       <c r="P23" s="9" t="inlineStr">
         <is>
-          <t>PT 0339050</t>
-        </is>
-      </c>
-      <c r="Q23" s="11" t="inlineStr"/>
+          <t>UM 03758004</t>
+        </is>
+      </c>
+      <c r="Q23" s="11" t="inlineStr">
+        <is>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3845467/3883533/77671008-6a79-4442-bbd3-dc2cfb091ca8?preview=true</t>
+        </is>
+      </c>
       <c r="R23" s="11" t="inlineStr">
         <is>
-          <t>Kitob tuman 1-son texnikumi</t>
+          <t>69-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S23" s="12" t="inlineStr">
         <is>
-          <t>Diplom</t>
+          <t>Shahodatnoma</t>
         </is>
       </c>
       <c r="T23" s="12" t="inlineStr">
@@ -28575,7 +28575,7 @@
       <c r="V23" s="11" t="inlineStr"/>
       <c r="W23" s="8" t="inlineStr">
         <is>
-          <t>Pasport: MOS</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="X23" s="7" t="inlineStr">
@@ -28595,7 +28595,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Temirova Rushana</t>
+          <t>Shukurova Zilola</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -28605,43 +28605,47 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>172</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-10 00:00:00</t>
+          <t>2026-09-02 00:00:00</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Sarvarovna</t>
+          <t>Farxod qizi</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Temirova Rushana Sarvarovna</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr"/>
+          <t>Shukurova Zilola Farxod qizi</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Shukurova Zilola Farxod qizi</t>
+        </is>
+      </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>AD9123776</t>
+          <t>AE1059205</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>60709085590113</t>
+          <t>60610085590150</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>23.10.2024</t>
+          <t>07.01.2025</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>07.09.2008</t>
+          <t>06.10.2008</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
@@ -28651,23 +28655,23 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>Mavjud</t>
+          <t>Shukurova Zilola Farhod qizi</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>UM 03755349</t>
+          <t>PT 0339050</t>
         </is>
       </c>
       <c r="Q24" s="4" t="inlineStr"/>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>Qashqadaryo viloyati, Shahrisabz tumani 61-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Kitob tuman 1-son texnikumi</t>
         </is>
       </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="T24" s="5" t="inlineStr">
@@ -28675,15 +28679,15 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="U24" s="17" t="inlineStr">
-        <is>
-          <t>FAYL_YOQ</t>
+      <c r="U24" s="7" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
         </is>
       </c>
       <c r="V24" s="4" t="inlineStr"/>
-      <c r="W24" s="15" t="inlineStr">
-        <is>
-          <t>TEKSHIRILMAGAN</t>
+      <c r="W24" s="8" t="inlineStr">
+        <is>
+          <t>Pasport: MOS</t>
         </is>
       </c>
       <c r="X24" s="7" t="inlineStr">
@@ -28703,7 +28707,7 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Toshpo'latova Asila</t>
+          <t>Temirova Rushana</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -28713,47 +28717,43 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>299</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>2026-09-02 00:00:00</t>
+          <t>2026-09-10 00:00:00</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>Akmal qizi</t>
+          <t>Sarvarovna</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Toshpo'latova Asila Akmal qizi</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>Toshpo'latova Asila Akmal qizi</t>
-        </is>
-      </c>
+          <t>Temirova Rushana Sarvarovna</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="12" t="inlineStr">
         <is>
-          <t>AE3444231</t>
+          <t>AD9123776</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>61709085590015</t>
+          <t>60709085590113</t>
         </is>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>18.07.2025</t>
+          <t>23.10.2024</t>
         </is>
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>17.09.2008</t>
+          <t>07.09.2008</t>
         </is>
       </c>
       <c r="N25" s="12" t="inlineStr">
@@ -28763,22 +28763,18 @@
       </c>
       <c r="O25" s="11" t="inlineStr">
         <is>
-          <t>Toshpo'latova Asila Akmal qizi</t>
+          <t>Mavjud</t>
         </is>
       </c>
       <c r="P25" s="9" t="inlineStr">
         <is>
-          <t>UM 03754061</t>
-        </is>
-      </c>
-      <c r="Q25" s="11" t="inlineStr">
-        <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3751197/3334326/3e3c9f4c-9b94-4ee1-9e1c-98c316a7d2dc?preview=true</t>
-        </is>
-      </c>
+          <t>UM 03755349</t>
+        </is>
+      </c>
+      <c r="Q25" s="11" t="inlineStr"/>
       <c r="R25" s="11" t="inlineStr">
         <is>
-          <t>26-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Qashqadaryo viloyati, Shahrisabz tumani 61-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S25" s="12" t="inlineStr">
@@ -28791,15 +28787,15 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="U25" s="7" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
+      <c r="U25" s="17" t="inlineStr">
+        <is>
+          <t>FAYL_YOQ</t>
         </is>
       </c>
       <c r="V25" s="11" t="inlineStr"/>
-      <c r="W25" s="8" t="inlineStr">
-        <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+      <c r="W25" s="15" t="inlineStr">
+        <is>
+          <t>TEKSHIRILMAGAN</t>
         </is>
       </c>
       <c r="X25" s="7" t="inlineStr">
@@ -28819,93 +28815,103 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Umirova Sevinch</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr"/>
+          <t>Toshpo'latova Asila</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>298</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>46275</v>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-02 00:00:00</t>
+        </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Avlayor qizi</t>
+          <t>Akmal qizi</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Umirova Sevinch Avlayor qizi</t>
+          <t>Toshpo'latova Asila Akmal qizi</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Umirova Sevinch Avlayor qizi</t>
+          <t>Toshpo'latova Asila Akmal qizi</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>AD1671106</t>
+          <t>AE3444231</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>60906055720101</t>
+          <t>61709085590015</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>18.08.2022</t>
+          <t>18.07.2025</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>09.06.2005</t>
+          <t>17.09.2008</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>Chiroqchi tumani</t>
-        </is>
-      </c>
-      <c r="O26" s="4" t="inlineStr"/>
+          <t>Shahrisabz tumani</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Toshpo'latova Asila Akmal qizi</t>
+        </is>
+      </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>UM 01891594</t>
-        </is>
-      </c>
-      <c r="Q26" s="4" t="inlineStr"/>
+          <t>UM 03754061</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3751197/3334326/3e3c9f4c-9b94-4ee1-9e1c-98c316a7d2dc?preview=true</t>
+        </is>
+      </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>42-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>26-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>ID-karta</t>
+          <t>Shahodatnoma</t>
         </is>
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="U26" s="16" t="inlineStr">
-        <is>
-          <t>CHALA</t>
-        </is>
-      </c>
-      <c r="V26" s="4" t="inlineStr">
-        <is>
-          <t>Pasportning orqa tomoni yo'q (JSHSHIR ko'rinmagan)</t>
-        </is>
-      </c>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U26" s="7" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V26" s="4" t="inlineStr"/>
       <c r="W26" s="8" t="inlineStr">
         <is>
-          <t>Pasport: MOS</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="X26" s="7" t="inlineStr">
@@ -28925,99 +28931,93 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Usmonova Yulduz</t>
+          <t>Umirova Sevinch</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr"/>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>209</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>2026-09-02 00:00:00</t>
-        </is>
+          <t>298</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="n">
+        <v>46275</v>
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Nu'mon qizi</t>
+          <t>Avlayor qizi</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>Usmonova Yulduz Nu'mon qizi</t>
+          <t>Umirova Sevinch Avlayor qizi</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
-          <t>Usmonova Yulduz Nu'mon qizi</t>
+          <t>Umirova Sevinch Avlayor qizi</t>
         </is>
       </c>
       <c r="J27" s="12" t="inlineStr">
         <is>
-          <t>AD9589389</t>
+          <t>AD1671106</t>
         </is>
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>62112075680077</t>
+          <t>60906055720101</t>
         </is>
       </c>
       <c r="L27" s="12" t="inlineStr">
         <is>
-          <t>27.11.2024</t>
+          <t>18.08.2022</t>
         </is>
       </c>
       <c r="M27" s="12" t="inlineStr">
         <is>
-          <t>21.12.2007</t>
+          <t>09.06.2005</t>
         </is>
       </c>
       <c r="N27" s="12" t="inlineStr">
         <is>
-          <t>Kitob tumani</t>
-        </is>
-      </c>
-      <c r="O27" s="11" t="inlineStr">
-        <is>
-          <t>Usmonova Yulduz Nu'mon qizi</t>
-        </is>
-      </c>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="O27" s="11" t="inlineStr"/>
       <c r="P27" s="9" t="inlineStr">
         <is>
-          <t>UM 03273678</t>
-        </is>
-      </c>
-      <c r="Q27" s="11" t="inlineStr">
-        <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/2510609/2335994/5d45b8e4-a117-4e26-ab03-12eb3391bac3?preview=true</t>
-        </is>
-      </c>
+          <t>UM 01891594</t>
+        </is>
+      </c>
+      <c r="Q27" s="11" t="inlineStr"/>
       <c r="R27" s="11" t="inlineStr">
         <is>
-          <t>12-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>42-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S27" s="12" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>ID-karta</t>
         </is>
       </c>
       <c r="T27" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="U27" s="7" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
-        </is>
-      </c>
-      <c r="V27" s="11" t="inlineStr"/>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="U27" s="16" t="inlineStr">
+        <is>
+          <t>CHALA</t>
+        </is>
+      </c>
+      <c r="V27" s="11" t="inlineStr">
+        <is>
+          <t>Pasportning orqa tomoni yo'q (JSHSHIR ko'rinmagan)</t>
+        </is>
+      </c>
       <c r="W27" s="8" t="inlineStr">
         <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+          <t>Pasport: MOS</t>
         </is>
       </c>
       <c r="X27" s="7" t="inlineStr">
@@ -29037,17 +29037,13 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Xaydarova Iroda</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
+          <t>Usmonova Yulduz</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>209</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -29057,62 +29053,62 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Zarif qizi</t>
+          <t>Nu'mon qizi</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Xaydarova Iroda Zarif qizi</t>
+          <t>Usmonova Yulduz Nu'mon qizi</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Xaydarova Iroda Zarif qizi</t>
+          <t>Usmonova Yulduz Nu'mon qizi</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>AE4240266</t>
+          <t>AD9589389</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>61906085590032</t>
+          <t>62112075680077</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>27.11.2024</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>19.06.2008</t>
+          <t>21.12.2007</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Shahrisabz tumani</t>
+          <t>Kitob tumani</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>Xaydarova Iroda Zarif qizi</t>
+          <t>Usmonova Yulduz Nu'mon qizi</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>UM 03754068</t>
+          <t>UM 03273678</t>
         </is>
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3751211/3334984/ed85efd3-f963-438f-9075-a2496493f195?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/2510609/2335994/5d45b8e4-a117-4e26-ab03-12eb3391bac3?preview=true</t>
         </is>
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>26-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>12-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S28" s="5" t="inlineStr">
@@ -29122,7 +29118,7 @@
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
@@ -29153,7 +29149,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Xayrullayeva Umida</t>
+          <t>Xaydarova Iroda</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -29163,7 +29159,7 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>113</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
@@ -29173,37 +29169,37 @@
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>Safar qizi</t>
+          <t>Zarif qizi</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Xayrullayeva Umida Safar qizi</t>
+          <t>Xaydarova Iroda Zarif qizi</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>Xayrullayeva Umida Safar qizi</t>
+          <t>Xaydarova Iroda Zarif qizi</t>
         </is>
       </c>
       <c r="J29" s="12" t="inlineStr">
         <is>
-          <t>AD9786798</t>
+          <t>AE4240266</t>
         </is>
       </c>
       <c r="K29" s="9" t="inlineStr">
         <is>
-          <t>61911085590096</t>
+          <t>61906085590032</t>
         </is>
       </c>
       <c r="L29" s="12" t="inlineStr">
         <is>
-          <t>12.12.2024</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="M29" s="12" t="inlineStr">
         <is>
-          <t>19.11.2008</t>
+          <t>19.06.2008</t>
         </is>
       </c>
       <c r="N29" s="12" t="inlineStr">
@@ -29213,23 +29209,27 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>Xayrullayeva Umida Safar qizi</t>
+          <t>Xaydarova Iroda Zarif qizi</t>
         </is>
       </c>
       <c r="P29" s="9" t="inlineStr">
         <is>
-          <t>PT 0025701</t>
-        </is>
-      </c>
-      <c r="Q29" s="11" t="inlineStr"/>
+          <t>UM 03754068</t>
+        </is>
+      </c>
+      <c r="Q29" s="11" t="inlineStr">
+        <is>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3751211/3334984/ed85efd3-f963-438f-9075-a2496493f195?preview=true</t>
+        </is>
+      </c>
       <c r="R29" s="11" t="inlineStr">
         <is>
-          <t>Kitob tuman 1-son texnikumi</t>
+          <t>26-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S29" s="12" t="inlineStr">
         <is>
-          <t>Diplom</t>
+          <t>Shahodatnoma</t>
         </is>
       </c>
       <c r="T29" s="12" t="inlineStr">
@@ -29243,9 +29243,9 @@
         </is>
       </c>
       <c r="V29" s="11" t="inlineStr"/>
-      <c r="W29" s="15" t="inlineStr">
-        <is>
-          <t>TEKSHIRILMAGAN</t>
+      <c r="W29" s="8" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="X29" s="7" t="inlineStr">
@@ -29265,13 +29265,17 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Xolmamatova Shoxista</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr"/>
+          <t>Xayrullayeva Umida</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>116</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -29281,67 +29285,63 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Sobir qizi</t>
+          <t>Safar qizi</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Xolmamatova Shoxista Sobir qizi</t>
+          <t>Xayrullayeva Umida Safar qizi</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Xolmamatova Shoxista Sobir qizi</t>
+          <t>Xayrullayeva Umida Safar qizi</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>AE4328716</t>
+          <t>AD9786798</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>60201085720092</t>
+          <t>61911085590096</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>24.09.2025</t>
+          <t>12.12.2024</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>02.01.2008</t>
+          <t>19.11.2008</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Chiroqchi tumani</t>
+          <t>Shahrisabz tumani</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>Xolmamatova Shoxista Sobir qizi</t>
+          <t>Xayrullayeva Umida Safar qizi</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>UM 03718337</t>
-        </is>
-      </c>
-      <c r="Q30" s="4" t="inlineStr">
-        <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4160257/3908748/b21b95c1-e731-4c4b-978a-b67116d7e66e?preview=true</t>
-        </is>
-      </c>
+          <t>PT 0025701</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr"/>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>36-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Kitob tuman 1-son texnikumi</t>
         </is>
       </c>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="T30" s="5" t="inlineStr">
@@ -29354,14 +29354,10 @@
           <t>TOPILDI</t>
         </is>
       </c>
-      <c r="V30" s="4" t="inlineStr">
-        <is>
-          <t>Familiyasi Xolmamatova Shoxista Sobir qizi deb to'g'rilandi (#243)</t>
-        </is>
-      </c>
-      <c r="W30" s="8" t="inlineStr">
-        <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+      <c r="V30" s="4" t="inlineStr"/>
+      <c r="W30" s="15" t="inlineStr">
+        <is>
+          <t>TEKSHIRILMAGAN</t>
         </is>
       </c>
       <c r="X30" s="7" t="inlineStr">
@@ -29381,17 +29377,13 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Xolmaxmatova Sevinch</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
+          <t>Xolmamatova Shoxista</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr"/>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>243</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
@@ -29401,62 +29393,62 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>Isomiddin qizi</t>
+          <t>Sobir qizi</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>Xolmaxmatova Sevinch Isomiddin qizi</t>
+          <t>Xolmamatova Shoxista Sobir qizi</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
         <is>
-          <t>Xolmaxmatova Sevinch Isomiddin qizi</t>
+          <t>Xolmamatova Shoxista Sobir qizi</t>
         </is>
       </c>
       <c r="J31" s="12" t="inlineStr">
         <is>
-          <t>AE4729924</t>
+          <t>AE4328716</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
         <is>
-          <t>62511085730064</t>
+          <t>60201085720092</t>
         </is>
       </c>
       <c r="L31" s="12" t="inlineStr">
         <is>
-          <t>22.10.2025</t>
+          <t>24.09.2025</t>
         </is>
       </c>
       <c r="M31" s="12" t="inlineStr">
         <is>
-          <t>25.11.2008</t>
+          <t>02.01.2008</t>
         </is>
       </c>
       <c r="N31" s="12" t="inlineStr">
         <is>
-          <t>Yakkabog' tumani</t>
+          <t>Chiroqchi tumani</t>
         </is>
       </c>
       <c r="O31" s="11" t="inlineStr">
         <is>
-          <t>Xolmaxmatova Sevinch Isomiddin qizi</t>
+          <t>Xolmamatova Shoxista Sobir qizi</t>
         </is>
       </c>
       <c r="P31" s="9" t="inlineStr">
         <is>
-          <t>UM 03758009</t>
+          <t>UM 03718337</t>
         </is>
       </c>
       <c r="Q31" s="11" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3845465/3883622/6f79b318-a4e1-46cb-ab79-97546eb5163a?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4160257/3908748/b21b95c1-e731-4c4b-978a-b67116d7e66e?preview=true</t>
         </is>
       </c>
       <c r="R31" s="11" t="inlineStr">
         <is>
-          <t>69-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>36-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S31" s="12" t="inlineStr">
@@ -29474,7 +29466,11 @@
           <t>TOPILDI</t>
         </is>
       </c>
-      <c r="V31" s="11" t="inlineStr"/>
+      <c r="V31" s="11" t="inlineStr">
+        <is>
+          <t>Familiyasi Xolmamatova Shoxista Sobir qizi deb to'g'rilandi (#243)</t>
+        </is>
+      </c>
       <c r="W31" s="8" t="inlineStr">
         <is>
           <t>Pasport: MOS | Shahodatnoma: MOS</t>
@@ -29497,7 +29493,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Xurramova Lobar</t>
+          <t>Xolmaxmatova Sevinch</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -29507,7 +29503,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>108</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -29517,62 +29513,62 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Ural qizi</t>
+          <t>Isomiddin qizi</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Xurramova Lobar Ural qizi</t>
+          <t>Xolmaxmatova Sevinch Isomiddin qizi</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Xurramova Lobar Ural qizi</t>
+          <t>Xolmaxmatova Sevinch Isomiddin qizi</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>AE2656510</t>
+          <t>AE4729924</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>62508085680062</t>
+          <t>62511085730064</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>13.05.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>25.08.2008</t>
+          <t>25.11.2008</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Kitob tumani</t>
+          <t>Yakkabog' tumani</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>Xurramova Lobar Ural qizi</t>
+          <t>Xolmaxmatova Sevinch Isomiddin qizi</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>UM 03728374</t>
+          <t>UM 03758009</t>
         </is>
       </c>
       <c r="Q32" s="4" t="inlineStr">
         <is>
-          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4050114/3589063/4a1b655d-a1f1-4f07-8a33-02afae733dd7?preview=true</t>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3845465/3883622/6f79b318-a4e1-46cb-ab79-97546eb5163a?preview=true</t>
         </is>
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>12-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>69-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S32" s="5" t="inlineStr">
@@ -29613,89 +29609,205 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
+          <t>Xurramova Lobar</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Ural qizi</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>Xurramova Lobar Ural qizi</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>Xurramova Lobar Ural qizi</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>AE2656510</t>
+        </is>
+      </c>
+      <c r="K33" s="9" t="inlineStr">
+        <is>
+          <t>62508085680062</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>13.05.2025</t>
+        </is>
+      </c>
+      <c r="M33" s="12" t="inlineStr">
+        <is>
+          <t>25.08.2008</t>
+        </is>
+      </c>
+      <c r="N33" s="12" t="inlineStr">
+        <is>
+          <t>Kitob tumani</t>
+        </is>
+      </c>
+      <c r="O33" s="11" t="inlineStr">
+        <is>
+          <t>Xurramova Lobar Ural qizi</t>
+        </is>
+      </c>
+      <c r="P33" s="9" t="inlineStr">
+        <is>
+          <t>UM 03728374</t>
+        </is>
+      </c>
+      <c r="Q33" s="11" t="inlineStr">
+        <is>
+          <t>https://e-shahodatnoma.uz/api/public/getcertpdf/4050114/3589063/4a1b655d-a1f1-4f07-8a33-02afae733dd7?preview=true</t>
+        </is>
+      </c>
+      <c r="R33" s="11" t="inlineStr">
+        <is>
+          <t>12-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
+      <c r="S33" s="12" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="T33" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U33" s="7" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V33" s="11" t="inlineStr"/>
+      <c r="W33" s="8" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+        </is>
+      </c>
+      <c r="X33" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
           <t>Xurramova Sabina</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr"/>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Yuldosh qizi</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>Xurramova Sabina Yuldosh qizi</t>
         </is>
       </c>
-      <c r="I33" s="10" t="inlineStr"/>
-      <c r="J33" s="12" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>AC3081523</t>
         </is>
       </c>
-      <c r="K33" s="9" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>60803048230011</t>
         </is>
       </c>
-      <c r="L33" s="12" t="inlineStr">
+      <c r="L34" s="5" t="inlineStr">
         <is>
           <t>16.10.2020</t>
         </is>
       </c>
-      <c r="M33" s="12" t="inlineStr">
+      <c r="M34" s="5" t="inlineStr">
         <is>
           <t>08.03.2004</t>
         </is>
       </c>
-      <c r="N33" s="12" t="inlineStr"/>
-      <c r="O33" s="11" t="inlineStr">
+      <c r="N34" s="5" t="inlineStr"/>
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>Mavjud</t>
         </is>
       </c>
-      <c r="P33" s="9" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>UM 1315230</t>
         </is>
       </c>
-      <c r="Q33" s="11" t="inlineStr"/>
-      <c r="R33" s="11" t="inlineStr">
+      <c r="Q34" s="4" t="inlineStr"/>
+      <c r="R34" s="4" t="inlineStr">
         <is>
           <t>4-sonli umumiy o’rta ta’lim maktabi</t>
         </is>
       </c>
-      <c r="S33" s="12" t="inlineStr">
+      <c r="S34" s="5" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="T33" s="12" t="inlineStr">
+      <c r="T34" s="5" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="U33" s="12" t="inlineStr"/>
-      <c r="V33" s="11" t="inlineStr"/>
-      <c r="W33" s="15" t="inlineStr"/>
-      <c r="X33" s="16" t="inlineStr">
+      <c r="U34" s="5" t="inlineStr"/>
+      <c r="V34" s="4" t="inlineStr"/>
+      <c r="W34" s="15" t="inlineStr"/>
+      <c r="X34" s="16" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X33"/>
+  <autoFilter ref="A1:X34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -41148,283 +41260,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="35" customWidth="1" min="17" max="17"/>
-    <col width="35" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="40" customWidth="1" min="22" max="22"/>
-    <col width="28" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>T/R</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Guruh</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>I.F.O</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>To'lov statusi</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Shartnoma raqami</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sanasi</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Otasining ismi (Sharifi)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>To'liq F.I.SH</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Passport bo'yicha F.I.SH</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Passport / ID-karta (Seriya va raqam)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>JSHSHIR (PINFL)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Berilgan sanasi</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Tug'ilgan sanasi</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Tug'ilgan tumani</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Shahodatnoma bo'yicha F.I.SH</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Shahodatnoma / Diplom Seriyasi</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Shahodatnoma QR Havolasi (e-shahodatnoma.uz)</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Tugatgan o'qish joyi</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Ta'lim muassasasi turi</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Bitirgan yili</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Qidiruv holati (Status)</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Izoh va Eslatmalar (Notes)</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Ism mosligi (Pasport / Shahodatnoma)</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Operator Tasdig'i</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>26-07</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Murtazayeva Kamola</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29 00:00:00</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Jamoliddin qizi</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Murtazayeva Kamola Jamoliddin qizi</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Murtazayeva Kamola Jamoliddin qizi</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>AC1458884</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>42708915590028</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>04.11.2018</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>27.08.1991</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>Shahrisabz tumani</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>Murtazayeva Kamola Jamoliddin qizi</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>O'r-Sh 0987579</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr"/>
-      <c r="R2" s="4" t="inlineStr">
-        <is>
-          <t>Ixtisoslashgan maktab</t>
-        </is>
-      </c>
-      <c r="S2" s="5" t="inlineStr">
-        <is>
-          <t>Shahodatnoma</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="n">
-        <v>2009</v>
-      </c>
-      <c r="U2" s="7" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>Otasining ismi 'Jamoliddin qizi' deb to'g'rilandi (#25)</t>
-        </is>
-      </c>
-      <c r="W2" s="8" t="inlineStr">
-        <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
-        </is>
-      </c>
-      <c r="X2" s="7" t="inlineStr">
-        <is>
-          <t>TASDIQLANDI</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:X2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>

</xml_diff>